<commit_message>
Add scalable fuzzy matcher with token index
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd6d1016bc1187ec/Proyecto GIA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\PycharmProjects\PlayWorth\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36C08D75-E207-4AF9-AD3A-0AB959074E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFDA0E6-478A-43B7-B20B-3FF7F260909E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9900" yWindow="5460" windowWidth="23535" windowHeight="13710" xr2:uid="{CF9629F7-1F1B-4C35-8467-92033BDE55BF}"/>
+    <workbookView xWindow="4995" yWindow="3630" windowWidth="28800" windowHeight="15345" xr2:uid="{CF9629F7-1F1B-4C35-8467-92033BDE55BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>The Witcher 3</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>game_name</t>
+  </si>
+  <si>
+    <t>Outer Wilds</t>
   </si>
 </sst>
 </file>
@@ -422,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F03D6BEC-E3FC-4415-9C5C-75DA198122DE}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
@@ -448,6 +451,11 @@
         <v>2</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>